<commit_message>
chore: add new asset
</commit_message>
<xml_diff>
--- a/assets/Form Pengujian UAT.xlsx
+++ b/assets/Form Pengujian UAT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ITERA\Kuliah Online\TA\Ackyras\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD3C1A28-0E48-4BC8-B978-9894B962428E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60BC812F-2800-40F4-A9AA-5812B0AF9EFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{EC2B1E6B-3C9F-4F9F-904A-4CD7C6F11A48}"/>
+    <workbookView xWindow="-27660" yWindow="660" windowWidth="23040" windowHeight="13560" xr2:uid="{EC2B1E6B-3C9F-4F9F-904A-4CD7C6F11A48}"/>
   </bookViews>
   <sheets>
     <sheet name="UAT" sheetId="7" r:id="rId1"/>
@@ -456,13 +456,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -495,11 +497,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -507,6 +504,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -835,28 +835,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
       <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
@@ -865,13 +865,13 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -881,9 +881,9 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="10"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="3" t="s">
         <v>11</v>
       </c>
@@ -891,9 +891,9 @@
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="10"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="11"/>
       <c r="D5" s="3" t="s">
         <v>12</v>
       </c>
@@ -901,9 +901,9 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="10"/>
+      <c r="A6" s="11"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="3" t="s">
         <v>13</v>
       </c>
@@ -911,9 +911,9 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="10"/>
+      <c r="A7" s="11"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="11"/>
       <c r="D7" s="3" t="s">
         <v>14</v>
       </c>
@@ -921,13 +921,13 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -937,9 +937,9 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="10"/>
+      <c r="A9" s="11"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="3" t="s">
         <v>17</v>
       </c>
@@ -947,9 +947,9 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="10"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="3" t="s">
         <v>18</v>
       </c>
@@ -957,9 +957,9 @@
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="10"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="3" t="s">
         <v>19</v>
       </c>
@@ -967,9 +967,9 @@
       <c r="F11" s="2"/>
     </row>
     <row r="12" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="10"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="11"/>
       <c r="D12" s="3" t="s">
         <v>20</v>
       </c>
@@ -977,13 +977,13 @@
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -993,9 +993,9 @@
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="10"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="10"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="3" t="s">
         <v>18</v>
       </c>
@@ -1003,9 +1003,9 @@
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="10"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="11"/>
       <c r="D15" s="3" t="s">
         <v>19</v>
       </c>
@@ -1013,9 +1013,9 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="10"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="10"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="3" t="s">
         <v>20</v>
       </c>
@@ -1023,13 +1023,13 @@
       <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -1039,9 +1039,9 @@
       <c r="F17" s="2"/>
     </row>
     <row r="18" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="10"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="11"/>
       <c r="D18" s="3" t="s">
         <v>25</v>
       </c>
@@ -1049,9 +1049,9 @@
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="10"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="11"/>
       <c r="D19" s="3" t="s">
         <v>26</v>
       </c>
@@ -1059,9 +1059,9 @@
       <c r="F19" s="2"/>
     </row>
     <row r="20" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="10"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="10"/>
+      <c r="A20" s="11"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="11"/>
       <c r="D20" s="3" t="s">
         <v>27</v>
       </c>
@@ -1069,13 +1069,13 @@
       <c r="F20" s="2"/>
     </row>
     <row r="21" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="11" t="s">
         <v>29</v>
       </c>
       <c r="D21" s="3" t="s">
@@ -1085,9 +1085,9 @@
       <c r="F21" s="2"/>
     </row>
     <row r="22" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="10"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="10"/>
+      <c r="A22" s="11"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="11"/>
       <c r="D22" s="3" t="s">
         <v>25</v>
       </c>
@@ -1095,9 +1095,9 @@
       <c r="F22" s="2"/>
     </row>
     <row r="23" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="10"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="10"/>
+      <c r="A23" s="11"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="11"/>
       <c r="D23" s="3" t="s">
         <v>26</v>
       </c>
@@ -1105,13 +1105,13 @@
       <c r="F23" s="2"/>
     </row>
     <row r="24" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D24" s="3" t="s">
@@ -1121,9 +1121,9 @@
       <c r="F24" s="2"/>
     </row>
     <row r="25" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="10"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="10"/>
+      <c r="A25" s="11"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="11"/>
       <c r="D25" s="3" t="s">
         <v>32</v>
       </c>
@@ -1131,9 +1131,9 @@
       <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="10"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="10"/>
+      <c r="A26" s="11"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="11"/>
       <c r="D26" s="3" t="s">
         <v>33</v>
       </c>
@@ -1141,9 +1141,9 @@
       <c r="F26" s="2"/>
     </row>
     <row r="27" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="10"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="10"/>
+      <c r="A27" s="11"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="11"/>
       <c r="D27" s="3" t="s">
         <v>34</v>
       </c>
@@ -1151,13 +1151,13 @@
       <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="11" t="s">
         <v>36</v>
       </c>
       <c r="D28" s="3" t="s">
@@ -1167,9 +1167,9 @@
       <c r="F28" s="2"/>
     </row>
     <row r="29" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="10"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="10"/>
+      <c r="A29" s="11"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="11"/>
       <c r="D29" s="3" t="s">
         <v>32</v>
       </c>
@@ -1177,9 +1177,9 @@
       <c r="F29" s="2"/>
     </row>
     <row r="30" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="10"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="10"/>
+      <c r="A30" s="11"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="11"/>
       <c r="D30" s="3" t="s">
         <v>33</v>
       </c>
@@ -1187,9 +1187,9 @@
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="10"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="10"/>
+      <c r="A31" s="11"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="11"/>
       <c r="D31" s="8" t="s">
         <v>34</v>
       </c>
@@ -1197,13 +1197,13 @@
       <c r="F31" s="2"/>
     </row>
     <row r="32" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D32" s="3" t="s">
@@ -1213,9 +1213,9 @@
       <c r="F32" s="2"/>
     </row>
     <row r="33" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="10"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="10"/>
+      <c r="A33" s="11"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="11"/>
       <c r="D33" s="3" t="s">
         <v>39</v>
       </c>
@@ -1223,9 +1223,9 @@
       <c r="F33" s="2"/>
     </row>
     <row r="34" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A34" s="10"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="10"/>
+      <c r="A34" s="11"/>
+      <c r="B34" s="12"/>
+      <c r="C34" s="11"/>
       <c r="D34" s="3" t="s">
         <v>40</v>
       </c>
@@ -1233,9 +1233,9 @@
       <c r="F34" s="2"/>
     </row>
     <row r="35" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="10"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="10"/>
+      <c r="A35" s="11"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="11"/>
       <c r="D35" s="3" t="s">
         <v>41</v>
       </c>
@@ -1243,13 +1243,13 @@
       <c r="F35" s="2"/>
     </row>
     <row r="36" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="C36" s="11" t="s">
         <v>29</v>
       </c>
       <c r="D36" s="3" t="s">
@@ -1259,9 +1259,9 @@
       <c r="F36" s="2"/>
     </row>
     <row r="37" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="10"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="10"/>
+      <c r="A37" s="11"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="11"/>
       <c r="D37" s="3" t="s">
         <v>39</v>
       </c>
@@ -1269,9 +1269,9 @@
       <c r="F37" s="2"/>
     </row>
     <row r="38" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="10"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="10"/>
+      <c r="A38" s="11"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="11"/>
       <c r="D38" s="3" t="s">
         <v>40</v>
       </c>
@@ -1279,9 +1279,9 @@
       <c r="F38" s="2"/>
     </row>
     <row r="39" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="10"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="10"/>
+      <c r="A39" s="11"/>
+      <c r="B39" s="12"/>
+      <c r="C39" s="11"/>
       <c r="D39" s="3" t="s">
         <v>41</v>
       </c>
@@ -1289,13 +1289,13 @@
       <c r="F39" s="2"/>
     </row>
     <row r="40" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="10" t="s">
+      <c r="A40" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="11" t="s">
         <v>36</v>
       </c>
       <c r="D40" s="3" t="s">
@@ -1305,9 +1305,9 @@
       <c r="F40" s="2"/>
     </row>
     <row r="41" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="10"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="10"/>
+      <c r="A41" s="11"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="11"/>
       <c r="D41" s="3" t="s">
         <v>45</v>
       </c>
@@ -1315,9 +1315,9 @@
       <c r="F41" s="2"/>
     </row>
     <row r="42" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A42" s="10"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="10"/>
+      <c r="A42" s="11"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="11"/>
       <c r="D42" s="3" t="s">
         <v>46</v>
       </c>
@@ -1325,9 +1325,9 @@
       <c r="F42" s="2"/>
     </row>
     <row r="43" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A43" s="10"/>
-      <c r="B43" s="11"/>
-      <c r="C43" s="10"/>
+      <c r="A43" s="11"/>
+      <c r="B43" s="12"/>
+      <c r="C43" s="11"/>
       <c r="D43" s="3" t="s">
         <v>47</v>
       </c>
@@ -1335,13 +1335,13 @@
       <c r="F43" s="2"/>
     </row>
     <row r="44" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A44" s="10" t="s">
+      <c r="A44" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="B44" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C44" s="11" t="s">
         <v>29</v>
       </c>
       <c r="D44" s="3" t="s">
@@ -1351,9 +1351,9 @@
       <c r="F44" s="2"/>
     </row>
     <row r="45" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A45" s="10"/>
-      <c r="B45" s="11"/>
-      <c r="C45" s="10"/>
+      <c r="A45" s="11"/>
+      <c r="B45" s="12"/>
+      <c r="C45" s="11"/>
       <c r="D45" s="3" t="s">
         <v>50</v>
       </c>
@@ -1361,9 +1361,9 @@
       <c r="F45" s="2"/>
     </row>
     <row r="46" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="10"/>
-      <c r="B46" s="11"/>
-      <c r="C46" s="10"/>
+      <c r="A46" s="11"/>
+      <c r="B46" s="12"/>
+      <c r="C46" s="11"/>
       <c r="D46" s="3" t="s">
         <v>51</v>
       </c>
@@ -1371,13 +1371,13 @@
       <c r="F46" s="2"/>
     </row>
     <row r="47" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A47" s="10" t="s">
+      <c r="A47" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B47" s="11" t="s">
+      <c r="B47" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="C47" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D47" s="3" t="s">
@@ -1387,9 +1387,9 @@
       <c r="F47" s="2"/>
     </row>
     <row r="48" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A48" s="10"/>
-      <c r="B48" s="11"/>
-      <c r="C48" s="10"/>
+      <c r="A48" s="11"/>
+      <c r="B48" s="12"/>
+      <c r="C48" s="11"/>
       <c r="D48" s="3" t="s">
         <v>54</v>
       </c>
@@ -1397,9 +1397,9 @@
       <c r="F48" s="2"/>
     </row>
     <row r="49" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A49" s="10"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="10"/>
+      <c r="A49" s="11"/>
+      <c r="B49" s="12"/>
+      <c r="C49" s="11"/>
       <c r="D49" s="3" t="s">
         <v>55</v>
       </c>
@@ -1407,13 +1407,13 @@
       <c r="F49" s="2"/>
     </row>
     <row r="50" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="10" t="s">
+      <c r="A50" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="11" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="3" t="s">
@@ -1423,9 +1423,9 @@
       <c r="F50" s="2"/>
     </row>
     <row r="51" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A51" s="10"/>
-      <c r="B51" s="11"/>
-      <c r="C51" s="10"/>
+      <c r="A51" s="11"/>
+      <c r="B51" s="12"/>
+      <c r="C51" s="11"/>
       <c r="D51" s="3" t="s">
         <v>58</v>
       </c>
@@ -1433,9 +1433,9 @@
       <c r="F51" s="2"/>
     </row>
     <row r="52" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A52" s="10"/>
-      <c r="B52" s="11"/>
-      <c r="C52" s="10"/>
+      <c r="A52" s="11"/>
+      <c r="B52" s="12"/>
+      <c r="C52" s="11"/>
       <c r="D52" s="3" t="s">
         <v>59</v>
       </c>
@@ -1443,11 +1443,11 @@
       <c r="F52" s="2"/>
     </row>
     <row r="53" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="9" t="s">
+      <c r="A53" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B53" s="9"/>
-      <c r="C53" s="9"/>
+      <c r="B53" s="13"/>
+      <c r="C53" s="13"/>
       <c r="D53" s="5">
         <f>COUNTA(D3:D52)</f>
         <v>50</v>
@@ -1456,11 +1456,11 @@
       <c r="F53" s="5"/>
     </row>
     <row r="54" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="9" t="s">
+      <c r="A54" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B54" s="9"/>
-      <c r="C54" s="9"/>
+      <c r="B54" s="13"/>
+      <c r="C54" s="13"/>
       <c r="D54" s="5">
         <f>COUNTA(D4:D53)</f>
         <v>50</v>
@@ -1477,6 +1477,36 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="46">
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="B50:B52"/>
+    <mergeCell ref="C50:C52"/>
+    <mergeCell ref="A40:A43"/>
+    <mergeCell ref="B40:B43"/>
+    <mergeCell ref="C40:C43"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="B32:B35"/>
+    <mergeCell ref="C32:C35"/>
+    <mergeCell ref="A36:A39"/>
+    <mergeCell ref="B36:B39"/>
+    <mergeCell ref="C36:C39"/>
+    <mergeCell ref="A24:A27"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="C24:C27"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="C28:C31"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="C8:C12"/>
     <mergeCell ref="A3:A7"/>
     <mergeCell ref="B3:B7"/>
     <mergeCell ref="C3:C7"/>
@@ -1484,11 +1514,6 @@
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="B8:B12"/>
-    <mergeCell ref="C8:C12"/>
     <mergeCell ref="A13:A16"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="C13:C16"/>
@@ -1498,31 +1523,6 @@
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="C21:C23"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="C24:C27"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="B28:B31"/>
-    <mergeCell ref="C28:C31"/>
-    <mergeCell ref="A32:A35"/>
-    <mergeCell ref="B32:B35"/>
-    <mergeCell ref="C32:C35"/>
-    <mergeCell ref="A36:A39"/>
-    <mergeCell ref="B36:B39"/>
-    <mergeCell ref="C36:C39"/>
-    <mergeCell ref="A40:A43"/>
-    <mergeCell ref="B40:B43"/>
-    <mergeCell ref="C40:C43"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="B50:B52"/>
-    <mergeCell ref="C50:C52"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="1.5748031496062993" right="1.1811023622047245" top="1.1811023622047245" bottom="1.1811023622047245" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -1550,28 +1550,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
       <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1580,13 +1580,13 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -1598,9 +1598,9 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="10"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1610,9 +1610,9 @@
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="10"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="11"/>
       <c r="D5" s="3" t="s">
         <v>12</v>
       </c>
@@ -1622,9 +1622,9 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="10"/>
+      <c r="A6" s="11"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="3" t="s">
         <v>13</v>
       </c>
@@ -1634,9 +1634,9 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="10"/>
+      <c r="A7" s="11"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="11"/>
       <c r="D7" s="3" t="s">
         <v>14</v>
       </c>
@@ -1646,13 +1646,13 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -1664,9 +1664,9 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="10"/>
+      <c r="A9" s="11"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="3" t="s">
         <v>17</v>
       </c>
@@ -1676,9 +1676,9 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="10"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="3" t="s">
         <v>18</v>
       </c>
@@ -1688,9 +1688,9 @@
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="10"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="3" t="s">
         <v>19</v>
       </c>
@@ -1700,9 +1700,9 @@
       <c r="F11" s="2"/>
     </row>
     <row r="12" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="10"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="11"/>
       <c r="D12" s="6" t="s">
         <v>20</v>
       </c>
@@ -1712,13 +1712,13 @@
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -1730,9 +1730,9 @@
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="10"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="10"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="3" t="s">
         <v>18</v>
       </c>
@@ -1742,9 +1742,9 @@
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="10"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="11"/>
       <c r="D15" s="3" t="s">
         <v>19</v>
       </c>
@@ -1754,9 +1754,9 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="10"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="10"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="7" t="s">
         <v>20</v>
       </c>
@@ -1766,11 +1766,11 @@
       <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="15"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="17"/>
       <c r="D17" s="5">
         <f>COUNTA(D3:D16)</f>
         <v>14</v>
@@ -1779,11 +1779,11 @@
       <c r="F17" s="5"/>
     </row>
     <row r="18" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="15"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="17"/>
       <c r="D18" s="5">
         <f>COUNTA(D4:D17)</f>
         <v>14</v>
@@ -1800,13 +1800,6 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="16">
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="C3:C7"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A17:C17"/>
@@ -1816,6 +1809,13 @@
     <mergeCell ref="A13:A16"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="C13:C16"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="1.5748031496062993" right="1.1811023622047245" top="1.1811023622047245" bottom="1.1811023622047245" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -1843,28 +1843,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
       <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1873,13 +1873,13 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -1891,9 +1891,9 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="17"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="17"/>
+      <c r="A4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="19"/>
       <c r="D4" s="3" t="s">
         <v>25</v>
       </c>
@@ -1903,9 +1903,9 @@
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="17"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="17"/>
+      <c r="A5" s="19"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="19"/>
       <c r="D5" s="3" t="s">
         <v>26</v>
       </c>
@@ -1915,9 +1915,9 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="18"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="18"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="20"/>
       <c r="D6" s="3" t="s">
         <v>27</v>
       </c>
@@ -1927,13 +1927,13 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="18" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -1945,9 +1945,9 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="17"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="17"/>
+      <c r="A8" s="19"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="19"/>
       <c r="D8" s="3" t="s">
         <v>25</v>
       </c>
@@ -1957,9 +1957,9 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="18"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="20"/>
       <c r="D9" s="3" t="s">
         <v>26</v>
       </c>
@@ -1969,11 +1969,11 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="15"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="17"/>
       <c r="D10" s="5">
         <f>COUNTA(D3:D9)</f>
         <v>7</v>
@@ -1982,11 +1982,11 @@
       <c r="F10" s="5"/>
     </row>
     <row r="11" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="15"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="17"/>
       <c r="D11" s="5">
         <f>COUNTA(D4:D10)</f>
         <v>7</v>
@@ -2003,11 +2003,6 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="13">
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A3:A6"/>
@@ -2016,6 +2011,11 @@
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="B7:B9"/>
     <mergeCell ref="C7:C9"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="1.5748031496062993" right="1.1811023622047245" top="1.1811023622047245" bottom="1.1811023622047245" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -2043,28 +2043,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
       <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
@@ -2073,13 +2073,13 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -2091,9 +2091,9 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="10"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="3" t="s">
         <v>32</v>
       </c>
@@ -2103,9 +2103,9 @@
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="10"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="11"/>
       <c r="D5" s="3" t="s">
         <v>33</v>
       </c>
@@ -2115,9 +2115,9 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="10"/>
+      <c r="A6" s="11"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="3" t="s">
         <v>34</v>
       </c>
@@ -2127,13 +2127,13 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="11" t="s">
         <v>36</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -2145,9 +2145,9 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="10"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="10"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="11"/>
       <c r="D8" s="3" t="s">
         <v>32</v>
       </c>
@@ -2157,9 +2157,9 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="10"/>
+      <c r="A9" s="11"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="3" t="s">
         <v>33</v>
       </c>
@@ -2169,9 +2169,9 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="10"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="3" t="s">
         <v>34</v>
       </c>
@@ -2181,13 +2181,13 @@
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="3" t="s">
@@ -2199,9 +2199,9 @@
       <c r="F11" s="2"/>
     </row>
     <row r="12" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="10"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="11"/>
       <c r="D12" s="3" t="s">
         <v>39</v>
       </c>
@@ -2211,9 +2211,9 @@
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="10"/>
+      <c r="A13" s="11"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="3" t="s">
         <v>40</v>
       </c>
@@ -2223,9 +2223,9 @@
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="10"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="10"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="3" t="s">
         <v>41</v>
       </c>
@@ -2235,13 +2235,13 @@
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="11" t="s">
         <v>29</v>
       </c>
       <c r="D15" s="3" t="s">
@@ -2253,9 +2253,9 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="10"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="10"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="3" t="s">
         <v>39</v>
       </c>
@@ -2265,9 +2265,9 @@
       <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="10"/>
+      <c r="A17" s="11"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="11"/>
       <c r="D17" s="3" t="s">
         <v>40</v>
       </c>
@@ -2277,9 +2277,9 @@
       <c r="F17" s="2"/>
     </row>
     <row r="18" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="10"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="11"/>
       <c r="D18" s="3" t="s">
         <v>41</v>
       </c>
@@ -2289,11 +2289,11 @@
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
       <c r="D19" s="5">
         <f>COUNTA(D3:D18)</f>
         <v>16</v>
@@ -2302,11 +2302,11 @@
       <c r="F19" s="5"/>
     </row>
     <row r="20" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
       <c r="D20" s="5">
         <f>COUNTA(D4:D19)</f>
         <v>16</v>
@@ -2323,11 +2323,6 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="19">
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="B3:B6"/>
@@ -2335,6 +2330,11 @@
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="B7:B10"/>
     <mergeCell ref="C7:C10"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A11:A14"/>
     <mergeCell ref="B11:B14"/>
@@ -2369,28 +2369,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
       <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
@@ -2399,13 +2399,13 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="18" t="s">
         <v>36</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -2417,9 +2417,9 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="17"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="17"/>
+      <c r="A4" s="19"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="19"/>
       <c r="D4" s="3" t="s">
         <v>45</v>
       </c>
@@ -2429,9 +2429,9 @@
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="17"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="17"/>
+      <c r="A5" s="19"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="19"/>
       <c r="D5" s="3" t="s">
         <v>46</v>
       </c>
@@ -2441,9 +2441,9 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="18"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="18"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="20"/>
       <c r="D6" s="3" t="s">
         <v>47</v>
       </c>
@@ -2453,13 +2453,13 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="18" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -2471,9 +2471,9 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="17"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="17"/>
+      <c r="A8" s="19"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="19"/>
       <c r="D8" s="3" t="s">
         <v>50</v>
       </c>
@@ -2483,9 +2483,9 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="18"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="20"/>
       <c r="D9" s="3" t="s">
         <v>51</v>
       </c>
@@ -2495,13 +2495,13 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -2513,9 +2513,9 @@
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="17"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="17"/>
+      <c r="A11" s="19"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="19"/>
       <c r="D11" s="3" t="s">
         <v>54</v>
       </c>
@@ -2525,9 +2525,9 @@
       <c r="F11" s="2"/>
     </row>
     <row r="12" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="18"/>
-      <c r="B12" s="21"/>
-      <c r="C12" s="18"/>
+      <c r="A12" s="20"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="20"/>
       <c r="D12" s="3" t="s">
         <v>55</v>
       </c>
@@ -2537,13 +2537,13 @@
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="18" t="s">
         <v>29</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -2555,9 +2555,9 @@
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="17"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="17"/>
+      <c r="A14" s="19"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="19"/>
       <c r="D14" s="3" t="s">
         <v>58</v>
       </c>
@@ -2567,9 +2567,9 @@
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="18"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="18"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="20"/>
       <c r="D15" s="3" t="s">
         <v>59</v>
       </c>
@@ -2579,11 +2579,11 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="15"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="17"/>
       <c r="D16" s="5">
         <f>COUNTA(D3:D15)</f>
         <v>13</v>
@@ -2592,11 +2592,11 @@
       <c r="F16" s="5"/>
     </row>
     <row r="17" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="15"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="17"/>
       <c r="D17" s="5">
         <f>COUNTA(D4:D16)</f>
         <v>13</v>
@@ -2613,11 +2613,6 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="19">
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="B3:B6"/>
@@ -2625,6 +2620,11 @@
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="B7:B9"/>
     <mergeCell ref="C7:C9"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="B10:B12"/>
@@ -2671,544 +2671,571 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
     </row>
     <row r="5" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="24"/>
-      <c r="B5" s="25"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="27"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="25"/>
+      <c r="J5" s="26"/>
     </row>
     <row r="6" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="24"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="27"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="26"/>
     </row>
     <row r="7" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="24"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="27"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="25"/>
+      <c r="J7" s="26"/>
     </row>
     <row r="8" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="24"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="27"/>
+      <c r="A8" s="10"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="25"/>
+      <c r="I8" s="25"/>
+      <c r="J8" s="26"/>
     </row>
     <row r="9" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="24"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="27"/>
+      <c r="A9" s="10"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="25"/>
+      <c r="J9" s="26"/>
     </row>
     <row r="10" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="24"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="27"/>
+      <c r="A10" s="10"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="26"/>
     </row>
     <row r="11" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="24"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="27"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="26"/>
     </row>
     <row r="12" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="24"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="27"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="25"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="26"/>
     </row>
     <row r="13" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="24"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="27"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="25"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="26"/>
     </row>
     <row r="14" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="24"/>
-      <c r="B14" s="25"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="27"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="26"/>
     </row>
     <row r="15" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="24"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="27"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="26"/>
     </row>
     <row r="16" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="24"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="27"/>
+      <c r="A16" s="10"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="26"/>
     </row>
     <row r="17" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="24"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="26"/>
-      <c r="J17" s="27"/>
+      <c r="A17" s="10"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="26"/>
     </row>
     <row r="18" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="24"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="27"/>
+      <c r="A18" s="10"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="26"/>
     </row>
     <row r="19" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="24"/>
-      <c r="B19" s="25"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="27"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="25"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="26"/>
     </row>
     <row r="20" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="24"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="27"/>
+      <c r="A20" s="10"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="26"/>
     </row>
     <row r="21" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="24"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="27"/>
+      <c r="A21" s="10"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="26"/>
     </row>
     <row r="22" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="24"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="26"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="27"/>
+      <c r="A22" s="10"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="25"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="25"/>
+      <c r="I22" s="25"/>
+      <c r="J22" s="26"/>
     </row>
     <row r="23" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="24"/>
-      <c r="B23" s="25"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26"/>
-      <c r="I23" s="26"/>
-      <c r="J23" s="27"/>
+      <c r="A23" s="10"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="26"/>
     </row>
     <row r="24" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="24"/>
-      <c r="B24" s="25"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="26"/>
-      <c r="I24" s="26"/>
-      <c r="J24" s="27"/>
+      <c r="A24" s="10"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="25"/>
+      <c r="I24" s="25"/>
+      <c r="J24" s="26"/>
     </row>
     <row r="25" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="24"/>
-      <c r="B25" s="25"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="26"/>
-      <c r="J25" s="27"/>
+      <c r="A25" s="10"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25"/>
+      <c r="I25" s="25"/>
+      <c r="J25" s="26"/>
     </row>
     <row r="26" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="24"/>
-      <c r="B26" s="25"/>
-      <c r="C26" s="26"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="26"/>
-      <c r="J26" s="27"/>
+      <c r="A26" s="10"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="25"/>
+      <c r="J26" s="26"/>
     </row>
     <row r="27" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="24"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="26"/>
-      <c r="J27" s="27"/>
+      <c r="A27" s="10"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="26"/>
     </row>
     <row r="28" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="24"/>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="27"/>
+      <c r="A28" s="10"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="26"/>
     </row>
     <row r="29" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="24"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="26"/>
-      <c r="J29" s="27"/>
+      <c r="A29" s="10"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="26"/>
     </row>
     <row r="30" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="24"/>
-      <c r="B30" s="25"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="26"/>
-      <c r="J30" s="27"/>
+      <c r="A30" s="10"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="26"/>
     </row>
     <row r="31" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="24"/>
-      <c r="B31" s="25"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="26"/>
-      <c r="J31" s="27"/>
+      <c r="A31" s="10"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="25"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="26"/>
     </row>
     <row r="32" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="24"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="27"/>
+      <c r="A32" s="10"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="25"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="26"/>
     </row>
     <row r="33" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="24"/>
-      <c r="B33" s="25"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="27"/>
+      <c r="A33" s="10"/>
+      <c r="B33" s="24"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="26"/>
     </row>
     <row r="34" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="24"/>
-      <c r="B34" s="25"/>
-      <c r="C34" s="26"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
-      <c r="J34" s="27"/>
+      <c r="A34" s="10"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="25"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="26"/>
     </row>
     <row r="35" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="24"/>
-      <c r="B35" s="25"/>
-      <c r="C35" s="26"/>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="26"/>
-      <c r="I35" s="26"/>
-      <c r="J35" s="27"/>
+      <c r="A35" s="10"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="25"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="25"/>
+      <c r="I35" s="25"/>
+      <c r="J35" s="26"/>
     </row>
     <row r="36" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="24"/>
-      <c r="B36" s="25"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="26"/>
-      <c r="J36" s="27"/>
+      <c r="A36" s="10"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25"/>
+      <c r="I36" s="25"/>
+      <c r="J36" s="26"/>
     </row>
     <row r="37" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="24"/>
-      <c r="B37" s="25"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="27"/>
+      <c r="A37" s="10"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="25"/>
+      <c r="F37" s="25"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="25"/>
+      <c r="I37" s="25"/>
+      <c r="J37" s="26"/>
     </row>
     <row r="38" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="24"/>
-      <c r="B38" s="25"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="26"/>
-      <c r="F38" s="26"/>
-      <c r="G38" s="26"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="26"/>
-      <c r="J38" s="27"/>
+      <c r="A38" s="10"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="25"/>
+      <c r="D38" s="25"/>
+      <c r="E38" s="25"/>
+      <c r="F38" s="25"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="25"/>
+      <c r="I38" s="25"/>
+      <c r="J38" s="26"/>
     </row>
     <row r="39" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="24"/>
-      <c r="B39" s="25"/>
-      <c r="C39" s="26"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="26"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="26"/>
-      <c r="J39" s="27"/>
+      <c r="A39" s="10"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="25"/>
+      <c r="D39" s="25"/>
+      <c r="E39" s="25"/>
+      <c r="F39" s="25"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="25"/>
+      <c r="I39" s="25"/>
+      <c r="J39" s="26"/>
     </row>
     <row r="40" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="24"/>
-      <c r="B40" s="25"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="26"/>
-      <c r="F40" s="26"/>
-      <c r="G40" s="26"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="26"/>
-      <c r="J40" s="27"/>
+      <c r="A40" s="10"/>
+      <c r="B40" s="24"/>
+      <c r="C40" s="25"/>
+      <c r="D40" s="25"/>
+      <c r="E40" s="25"/>
+      <c r="F40" s="25"/>
+      <c r="G40" s="25"/>
+      <c r="H40" s="25"/>
+      <c r="I40" s="25"/>
+      <c r="J40" s="26"/>
     </row>
     <row r="41" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="24"/>
-      <c r="B41" s="25"/>
-      <c r="C41" s="26"/>
-      <c r="D41" s="26"/>
-      <c r="E41" s="26"/>
-      <c r="F41" s="26"/>
-      <c r="G41" s="26"/>
-      <c r="H41" s="26"/>
-      <c r="I41" s="26"/>
-      <c r="J41" s="27"/>
+      <c r="A41" s="10"/>
+      <c r="B41" s="24"/>
+      <c r="C41" s="25"/>
+      <c r="D41" s="25"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="25"/>
+      <c r="G41" s="25"/>
+      <c r="H41" s="25"/>
+      <c r="I41" s="25"/>
+      <c r="J41" s="26"/>
     </row>
     <row r="42" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="24"/>
-      <c r="B42" s="25"/>
-      <c r="C42" s="26"/>
-      <c r="D42" s="26"/>
-      <c r="E42" s="26"/>
-      <c r="F42" s="26"/>
-      <c r="G42" s="26"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="26"/>
-      <c r="J42" s="27"/>
+      <c r="A42" s="10"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="25"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="25"/>
+      <c r="I42" s="25"/>
+      <c r="J42" s="26"/>
     </row>
     <row r="43" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="24"/>
-      <c r="B43" s="25"/>
-      <c r="C43" s="26"/>
-      <c r="D43" s="26"/>
-      <c r="E43" s="26"/>
-      <c r="F43" s="26"/>
-      <c r="G43" s="26"/>
-      <c r="H43" s="26"/>
-      <c r="I43" s="26"/>
-      <c r="J43" s="27"/>
+      <c r="A43" s="10"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="25"/>
+      <c r="D43" s="25"/>
+      <c r="E43" s="25"/>
+      <c r="F43" s="25"/>
+      <c r="G43" s="25"/>
+      <c r="H43" s="25"/>
+      <c r="I43" s="25"/>
+      <c r="J43" s="26"/>
     </row>
     <row r="44" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="24"/>
-      <c r="B44" s="25"/>
-      <c r="C44" s="26"/>
-      <c r="D44" s="26"/>
-      <c r="E44" s="26"/>
-      <c r="F44" s="26"/>
-      <c r="G44" s="26"/>
-      <c r="H44" s="26"/>
-      <c r="I44" s="26"/>
-      <c r="J44" s="27"/>
+      <c r="A44" s="10"/>
+      <c r="B44" s="24"/>
+      <c r="C44" s="25"/>
+      <c r="D44" s="25"/>
+      <c r="E44" s="25"/>
+      <c r="F44" s="25"/>
+      <c r="G44" s="25"/>
+      <c r="H44" s="25"/>
+      <c r="I44" s="25"/>
+      <c r="J44" s="26"/>
     </row>
     <row r="45" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="24"/>
-      <c r="B45" s="25"/>
-      <c r="C45" s="26"/>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="26"/>
-      <c r="I45" s="26"/>
-      <c r="J45" s="27"/>
+      <c r="A45" s="10"/>
+      <c r="B45" s="24"/>
+      <c r="C45" s="25"/>
+      <c r="D45" s="25"/>
+      <c r="E45" s="25"/>
+      <c r="F45" s="25"/>
+      <c r="G45" s="25"/>
+      <c r="H45" s="25"/>
+      <c r="I45" s="25"/>
+      <c r="J45" s="26"/>
     </row>
     <row r="46" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="24"/>
-      <c r="B46" s="25"/>
-      <c r="C46" s="26"/>
-      <c r="D46" s="26"/>
-      <c r="E46" s="26"/>
-      <c r="F46" s="26"/>
-      <c r="G46" s="26"/>
-      <c r="H46" s="26"/>
-      <c r="I46" s="26"/>
-      <c r="J46" s="27"/>
+      <c r="A46" s="10"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="25"/>
+      <c r="E46" s="25"/>
+      <c r="F46" s="25"/>
+      <c r="G46" s="25"/>
+      <c r="H46" s="25"/>
+      <c r="I46" s="25"/>
+      <c r="J46" s="26"/>
     </row>
     <row r="47" spans="1:10" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="24"/>
-      <c r="B47" s="25"/>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="26"/>
-      <c r="I47" s="26"/>
-      <c r="J47" s="27"/>
+      <c r="A47" s="10"/>
+      <c r="B47" s="24"/>
+      <c r="C47" s="25"/>
+      <c r="D47" s="25"/>
+      <c r="E47" s="25"/>
+      <c r="F47" s="25"/>
+      <c r="G47" s="25"/>
+      <c r="H47" s="25"/>
+      <c r="I47" s="25"/>
+      <c r="J47" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="B42:J42"/>
-    <mergeCell ref="B43:J43"/>
-    <mergeCell ref="B44:J44"/>
-    <mergeCell ref="B45:J45"/>
-    <mergeCell ref="B46:J46"/>
+    <mergeCell ref="B9:J9"/>
+    <mergeCell ref="B10:J10"/>
+    <mergeCell ref="B11:J11"/>
+    <mergeCell ref="B4:J4"/>
+    <mergeCell ref="B5:J5"/>
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="B8:J8"/>
+    <mergeCell ref="B23:J23"/>
+    <mergeCell ref="B12:J12"/>
+    <mergeCell ref="B13:J13"/>
+    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B16:J16"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="B19:J19"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="B22:J22"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="B25:J25"/>
+    <mergeCell ref="B26:J26"/>
+    <mergeCell ref="B27:J27"/>
+    <mergeCell ref="B28:J28"/>
+    <mergeCell ref="B29:J29"/>
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="B31:J31"/>
+    <mergeCell ref="B32:J32"/>
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="B34:J34"/>
     <mergeCell ref="B47:J47"/>
     <mergeCell ref="B36:J36"/>
     <mergeCell ref="B37:J37"/>
@@ -3216,38 +3243,11 @@
     <mergeCell ref="B39:J39"/>
     <mergeCell ref="B40:J40"/>
     <mergeCell ref="B41:J41"/>
-    <mergeCell ref="B30:J30"/>
-    <mergeCell ref="B31:J31"/>
-    <mergeCell ref="B32:J32"/>
-    <mergeCell ref="B33:J33"/>
-    <mergeCell ref="B34:J34"/>
-    <mergeCell ref="B35:J35"/>
-    <mergeCell ref="B24:J24"/>
-    <mergeCell ref="B25:J25"/>
-    <mergeCell ref="B26:J26"/>
-    <mergeCell ref="B27:J27"/>
-    <mergeCell ref="B28:J28"/>
-    <mergeCell ref="B29:J29"/>
-    <mergeCell ref="B18:J18"/>
-    <mergeCell ref="B19:J19"/>
-    <mergeCell ref="B20:J20"/>
-    <mergeCell ref="B21:J21"/>
-    <mergeCell ref="B22:J22"/>
-    <mergeCell ref="B23:J23"/>
-    <mergeCell ref="B12:J12"/>
-    <mergeCell ref="B13:J13"/>
-    <mergeCell ref="B14:J14"/>
-    <mergeCell ref="B15:J15"/>
-    <mergeCell ref="B16:J16"/>
-    <mergeCell ref="B17:J17"/>
-    <mergeCell ref="B4:J4"/>
-    <mergeCell ref="B5:J5"/>
-    <mergeCell ref="B6:J6"/>
-    <mergeCell ref="B7:J7"/>
-    <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B9:J9"/>
-    <mergeCell ref="B10:J10"/>
-    <mergeCell ref="B11:J11"/>
+    <mergeCell ref="B42:J42"/>
+    <mergeCell ref="B43:J43"/>
+    <mergeCell ref="B44:J44"/>
+    <mergeCell ref="B45:J45"/>
+    <mergeCell ref="B46:J46"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>